<commit_message>
data: log county officeholder backfill in MS_Municipalities.xlsx (issue #36)
Marks the SOS directory source as USED in the Sources sheet, notes on
every Counties row that officeholders are now seeded in the repo data
files (per the workbook's own design, not duplicated into this sheet),
updates the README coverage line, and adds a Status Log entry for
commit a89592ede.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ve3atLELtBgTmGubX2xjUz
</commit_message>
<xml_diff>
--- a/reference/MS Rolling Audit/MS_Municipalities.xlsx
+++ b/reference/MS Rolling Audit/MS_Municipalities.xlsx
@@ -491,6 +491,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="9">
       <c r="A4" s="12" t="inlineStr">
         <is>
@@ -555,7 +556,7 @@
       </c>
       <c r="C7" s="13" t="inlineStr">
         <is>
-          <t>82 counties; official county websites = Needs Research.</t>
+          <t>82 counties; official county websites = Needs Research. Elected officeholders (13 office types, 1,825 people) seeded in repo data files.</t>
         </is>
       </c>
     </row>
@@ -16691,7 +16692,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F2" s="14" t="n"/>
+      <c r="F2" s="14" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="15" customHeight="1" s="9">
       <c r="A3" s="13" t="inlineStr">
@@ -16717,7 +16722,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F3" s="13" t="n"/>
+      <c r="F3" s="13" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="15" customHeight="1" s="9">
       <c r="A4" s="14" t="inlineStr">
@@ -16743,7 +16752,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F4" s="14" t="n"/>
+      <c r="F4" s="14" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="9">
       <c r="A5" s="13" t="inlineStr">
@@ -16769,7 +16782,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F5" s="13" t="n"/>
+      <c r="F5" s="13" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="9">
       <c r="A6" s="14" t="inlineStr">
@@ -16795,7 +16812,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F6" s="14" t="n"/>
+      <c r="F6" s="14" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="9">
       <c r="A7" s="13" t="inlineStr">
@@ -16821,7 +16842,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F7" s="13" t="n"/>
+      <c r="F7" s="13" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="9">
       <c r="A8" s="14" t="inlineStr">
@@ -16847,7 +16872,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F8" s="14" t="n"/>
+      <c r="F8" s="14" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="9">
       <c r="A9" s="13" t="inlineStr">
@@ -16873,7 +16902,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F9" s="13" t="n"/>
+      <c r="F9" s="13" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="9">
       <c r="A10" s="14" t="inlineStr">
@@ -16899,7 +16932,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F10" s="14" t="n"/>
+      <c r="F10" s="14" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="9">
       <c r="A11" s="13" t="inlineStr">
@@ -16925,7 +16962,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F11" s="13" t="n"/>
+      <c r="F11" s="13" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="9">
       <c r="A12" s="14" t="inlineStr">
@@ -16951,7 +16992,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F12" s="14" t="n"/>
+      <c r="F12" s="14" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="9">
       <c r="A13" s="13" t="inlineStr">
@@ -16977,7 +17022,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F13" s="13" t="n"/>
+      <c r="F13" s="13" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="9">
       <c r="A14" s="14" t="inlineStr">
@@ -17003,7 +17052,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F14" s="14" t="n"/>
+      <c r="F14" s="14" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="9">
       <c r="A15" s="13" t="inlineStr">
@@ -17029,7 +17082,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F15" s="13" t="n"/>
+      <c r="F15" s="13" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="9">
       <c r="A16" s="14" t="inlineStr">
@@ -17055,7 +17112,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F16" s="14" t="n"/>
+      <c r="F16" s="14" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="9">
       <c r="A17" s="13" t="inlineStr">
@@ -17081,7 +17142,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F17" s="13" t="n"/>
+      <c r="F17" s="13" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="9">
       <c r="A18" s="14" t="inlineStr">
@@ -17107,7 +17172,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F18" s="14" t="n"/>
+      <c r="F18" s="14" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="15" customHeight="1" s="9">
       <c r="A19" s="13" t="inlineStr">
@@ -17133,7 +17202,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F19" s="13" t="n"/>
+      <c r="F19" s="13" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="9">
       <c r="A20" s="14" t="inlineStr">
@@ -17159,7 +17232,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F20" s="14" t="n"/>
+      <c r="F20" s="14" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="15" customHeight="1" s="9">
       <c r="A21" s="13" t="inlineStr">
@@ -17185,7 +17262,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F21" s="13" t="n"/>
+      <c r="F21" s="13" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="15" customHeight="1" s="9">
       <c r="A22" s="14" t="inlineStr">
@@ -17211,7 +17292,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F22" s="14" t="n"/>
+      <c r="F22" s="14" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="15" customHeight="1" s="9">
       <c r="A23" s="13" t="inlineStr">
@@ -17237,7 +17322,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F23" s="13" t="n"/>
+      <c r="F23" s="13" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="15" customHeight="1" s="9">
       <c r="A24" s="14" t="inlineStr">
@@ -17263,7 +17352,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F24" s="14" t="n"/>
+      <c r="F24" s="14" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="15" customHeight="1" s="9">
       <c r="A25" s="13" t="inlineStr">
@@ -17289,7 +17382,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F25" s="13" t="n"/>
+      <c r="F25" s="13" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="15" customHeight="1" s="9">
       <c r="A26" s="14" t="inlineStr">
@@ -17315,7 +17412,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F26" s="14" t="n"/>
+      <c r="F26" s="14" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="15" customHeight="1" s="9">
       <c r="A27" s="13" t="inlineStr">
@@ -17341,7 +17442,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F27" s="13" t="n"/>
+      <c r="F27" s="13" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="15" customHeight="1" s="9">
       <c r="A28" s="14" t="inlineStr">
@@ -17367,7 +17472,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F28" s="14" t="n"/>
+      <c r="F28" s="14" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="15" customHeight="1" s="9">
       <c r="A29" s="13" t="inlineStr">
@@ -17393,7 +17502,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F29" s="13" t="n"/>
+      <c r="F29" s="13" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="15" customHeight="1" s="9">
       <c r="A30" s="14" t="inlineStr">
@@ -17419,7 +17532,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F30" s="14" t="n"/>
+      <c r="F30" s="14" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="15" customHeight="1" s="9">
       <c r="A31" s="13" t="inlineStr">
@@ -17445,7 +17562,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F31" s="13" t="n"/>
+      <c r="F31" s="13" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="15" customHeight="1" s="9">
       <c r="A32" s="14" t="inlineStr">
@@ -17471,7 +17592,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F32" s="14" t="n"/>
+      <c r="F32" s="14" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="15" customHeight="1" s="9">
       <c r="A33" s="13" t="inlineStr">
@@ -17497,7 +17622,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F33" s="13" t="n"/>
+      <c r="F33" s="13" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="15" customHeight="1" s="9">
       <c r="A34" s="14" t="inlineStr">
@@ -17523,7 +17652,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F34" s="14" t="n"/>
+      <c r="F34" s="14" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="15" customHeight="1" s="9">
       <c r="A35" s="13" t="inlineStr">
@@ -17549,7 +17682,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F35" s="13" t="n"/>
+      <c r="F35" s="13" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="15" customHeight="1" s="9">
       <c r="A36" s="14" t="inlineStr">
@@ -17575,7 +17712,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F36" s="14" t="n"/>
+      <c r="F36" s="14" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="15" customHeight="1" s="9">
       <c r="A37" s="13" t="inlineStr">
@@ -17601,7 +17742,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F37" s="13" t="n"/>
+      <c r="F37" s="13" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="15" customHeight="1" s="9">
       <c r="A38" s="14" t="inlineStr">
@@ -17627,7 +17772,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F38" s="14" t="n"/>
+      <c r="F38" s="14" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="15" customHeight="1" s="9">
       <c r="A39" s="13" t="inlineStr">
@@ -17653,7 +17802,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F39" s="13" t="n"/>
+      <c r="F39" s="13" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="15" customHeight="1" s="9">
       <c r="A40" s="14" t="inlineStr">
@@ -17679,7 +17832,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F40" s="14" t="n"/>
+      <c r="F40" s="14" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="15" customHeight="1" s="9">
       <c r="A41" s="13" t="inlineStr">
@@ -17705,7 +17862,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F41" s="13" t="n"/>
+      <c r="F41" s="13" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="15" customHeight="1" s="9">
       <c r="A42" s="14" t="inlineStr">
@@ -17731,7 +17892,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F42" s="14" t="n"/>
+      <c r="F42" s="14" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="15" customHeight="1" s="9">
       <c r="A43" s="13" t="inlineStr">
@@ -17757,7 +17922,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F43" s="13" t="n"/>
+      <c r="F43" s="13" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="15" customHeight="1" s="9">
       <c r="A44" s="14" t="inlineStr">
@@ -17783,7 +17952,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F44" s="14" t="n"/>
+      <c r="F44" s="14" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="15" customHeight="1" s="9">
       <c r="A45" s="13" t="inlineStr">
@@ -17809,7 +17982,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F45" s="13" t="n"/>
+      <c r="F45" s="13" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="15" customHeight="1" s="9">
       <c r="A46" s="14" t="inlineStr">
@@ -17835,7 +18012,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F46" s="14" t="n"/>
+      <c r="F46" s="14" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="15" customHeight="1" s="9">
       <c r="A47" s="13" t="inlineStr">
@@ -17861,7 +18042,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F47" s="13" t="n"/>
+      <c r="F47" s="13" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="15" customHeight="1" s="9">
       <c r="A48" s="14" t="inlineStr">
@@ -17887,7 +18072,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F48" s="14" t="n"/>
+      <c r="F48" s="14" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="15" customHeight="1" s="9">
       <c r="A49" s="13" t="inlineStr">
@@ -17913,7 +18102,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F49" s="13" t="n"/>
+      <c r="F49" s="13" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="15" customHeight="1" s="9">
       <c r="A50" s="14" t="inlineStr">
@@ -17939,7 +18132,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F50" s="14" t="n"/>
+      <c r="F50" s="14" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="15" customHeight="1" s="9">
       <c r="A51" s="13" t="inlineStr">
@@ -17965,7 +18162,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F51" s="13" t="n"/>
+      <c r="F51" s="13" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="15" customHeight="1" s="9">
       <c r="A52" s="14" t="inlineStr">
@@ -17991,7 +18192,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F52" s="14" t="n"/>
+      <c r="F52" s="14" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="15" customHeight="1" s="9">
       <c r="A53" s="13" t="inlineStr">
@@ -18017,7 +18222,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F53" s="13" t="n"/>
+      <c r="F53" s="13" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="15" customHeight="1" s="9">
       <c r="A54" s="14" t="inlineStr">
@@ -18043,7 +18252,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F54" s="14" t="n"/>
+      <c r="F54" s="14" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="15" customHeight="1" s="9">
       <c r="A55" s="13" t="inlineStr">
@@ -18069,7 +18282,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F55" s="13" t="n"/>
+      <c r="F55" s="13" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="15" customHeight="1" s="9">
       <c r="A56" s="14" t="inlineStr">
@@ -18095,7 +18312,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F56" s="14" t="n"/>
+      <c r="F56" s="14" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="15" customHeight="1" s="9">
       <c r="A57" s="13" t="inlineStr">
@@ -18121,7 +18342,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F57" s="13" t="n"/>
+      <c r="F57" s="13" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="58" ht="15" customHeight="1" s="9">
       <c r="A58" s="14" t="inlineStr">
@@ -18147,7 +18372,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F58" s="14" t="n"/>
+      <c r="F58" s="14" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="59" ht="15" customHeight="1" s="9">
       <c r="A59" s="13" t="inlineStr">
@@ -18173,7 +18402,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F59" s="13" t="n"/>
+      <c r="F59" s="13" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="60" ht="15" customHeight="1" s="9">
       <c r="A60" s="14" t="inlineStr">
@@ -18199,7 +18432,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F60" s="14" t="n"/>
+      <c r="F60" s="14" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="61" ht="15" customHeight="1" s="9">
       <c r="A61" s="13" t="inlineStr">
@@ -18225,7 +18462,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F61" s="13" t="n"/>
+      <c r="F61" s="13" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="62" ht="15" customHeight="1" s="9">
       <c r="A62" s="14" t="inlineStr">
@@ -18251,7 +18492,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F62" s="14" t="n"/>
+      <c r="F62" s="14" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="63" ht="15" customHeight="1" s="9">
       <c r="A63" s="13" t="inlineStr">
@@ -18277,7 +18522,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F63" s="13" t="n"/>
+      <c r="F63" s="13" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="15" customHeight="1" s="9">
       <c r="A64" s="14" t="inlineStr">
@@ -18303,7 +18552,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F64" s="14" t="n"/>
+      <c r="F64" s="14" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="65" ht="15" customHeight="1" s="9">
       <c r="A65" s="13" t="inlineStr">
@@ -18329,7 +18582,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F65" s="13" t="n"/>
+      <c r="F65" s="13" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="66" ht="15" customHeight="1" s="9">
       <c r="A66" s="14" t="inlineStr">
@@ -18355,7 +18612,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F66" s="14" t="n"/>
+      <c r="F66" s="14" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="67" ht="15" customHeight="1" s="9">
       <c r="A67" s="13" t="inlineStr">
@@ -18381,7 +18642,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F67" s="13" t="n"/>
+      <c r="F67" s="13" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="68" ht="15" customHeight="1" s="9">
       <c r="A68" s="14" t="inlineStr">
@@ -18407,7 +18672,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F68" s="14" t="n"/>
+      <c r="F68" s="14" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="69" ht="15" customHeight="1" s="9">
       <c r="A69" s="13" t="inlineStr">
@@ -18433,7 +18702,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F69" s="13" t="n"/>
+      <c r="F69" s="13" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="70" ht="15" customHeight="1" s="9">
       <c r="A70" s="14" t="inlineStr">
@@ -18459,7 +18732,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F70" s="14" t="n"/>
+      <c r="F70" s="14" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="71" ht="15" customHeight="1" s="9">
       <c r="A71" s="13" t="inlineStr">
@@ -18485,7 +18762,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F71" s="13" t="n"/>
+      <c r="F71" s="13" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="72" ht="15" customHeight="1" s="9">
       <c r="A72" s="14" t="inlineStr">
@@ -18511,7 +18792,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F72" s="14" t="n"/>
+      <c r="F72" s="14" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="73" ht="15" customHeight="1" s="9">
       <c r="A73" s="13" t="inlineStr">
@@ -18537,7 +18822,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F73" s="13" t="n"/>
+      <c r="F73" s="13" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="74" ht="15" customHeight="1" s="9">
       <c r="A74" s="14" t="inlineStr">
@@ -18563,7 +18852,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F74" s="14" t="n"/>
+      <c r="F74" s="14" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="75" ht="15" customHeight="1" s="9">
       <c r="A75" s="13" t="inlineStr">
@@ -18589,7 +18882,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F75" s="13" t="n"/>
+      <c r="F75" s="13" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="76" ht="15" customHeight="1" s="9">
       <c r="A76" s="14" t="inlineStr">
@@ -18615,7 +18912,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F76" s="14" t="n"/>
+      <c r="F76" s="14" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="77" ht="15" customHeight="1" s="9">
       <c r="A77" s="13" t="inlineStr">
@@ -18641,7 +18942,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F77" s="13" t="n"/>
+      <c r="F77" s="13" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="78" ht="15" customHeight="1" s="9">
       <c r="A78" s="14" t="inlineStr">
@@ -18667,7 +18972,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F78" s="14" t="n"/>
+      <c r="F78" s="14" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="79" ht="15" customHeight="1" s="9">
       <c r="A79" s="13" t="inlineStr">
@@ -18693,7 +19002,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F79" s="13" t="n"/>
+      <c r="F79" s="13" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="80" ht="15" customHeight="1" s="9">
       <c r="A80" s="14" t="inlineStr">
@@ -18719,7 +19032,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F80" s="14" t="n"/>
+      <c r="F80" s="14" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="81" ht="15" customHeight="1" s="9">
       <c r="A81" s="13" t="inlineStr">
@@ -18745,7 +19062,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F81" s="13" t="n"/>
+      <c r="F81" s="13" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="82" ht="15" customHeight="1" s="9">
       <c r="A82" s="14" t="inlineStr">
@@ -18771,7 +19092,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F82" s="14" t="n"/>
+      <c r="F82" s="14" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
     <row r="83" ht="15" customHeight="1" s="9">
       <c r="A83" s="13" t="inlineStr">
@@ -18797,7 +19122,11 @@
           <t>Needs Research</t>
         </is>
       </c>
-      <c r="F83" s="13" t="n"/>
+      <c r="F83" s="13" t="inlineStr">
+        <is>
+          <t>Elected officeholders (13 office types) seeded in repo data/us/ms/{organizations,posts,people,memberships}/county/ -- see issue #36.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:F83"/>
@@ -19291,12 +19620,12 @@
       </c>
       <c r="G5" s="13" t="inlineStr">
         <is>
-          <t>TODO — form &amp; officeholders</t>
+          <t>USED — county officeholders (2026 directory)</t>
         </is>
       </c>
       <c r="H5" s="13" t="inlineStr">
         <is>
-          <t>Check for a downloadable municipal directory / elections API.</t>
+          <t>County Offices and Directory (2026) PDF used to seed 82 counties' elected officeholders into repo data files (see Counties sheet note + Status Log). Municipal charter/officeholder backfill from this source is still TODO.</t>
         </is>
       </c>
     </row>
@@ -19439,7 +19768,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="12" customWidth="1" style="8" min="1" max="1"/>
@@ -19558,27 +19887,54 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>Completed the City Website backfill pass for all 299 municipalities via 3 parallel research agents covering the 150 towns still unresolved after the MML scrape + pattern-guess passes. 40 more official websites found and confirmed Mississippi-specific (27 high confidence, 13 medium confidence -- flagged with a verification-obstacle note in Notes, e.g. SSL cert errors or a subdomain of a county's own site, during research; treat as needing a human spot-check before treating as fully authoritative). The remaining 110 were individually researched and confirmed to have no locatable official government website -- Status marked accordingly so future sessions know these were checked, not skipped. One (Shubuta) corrected from the MML/pattern-guess passes' 'no website' finding after the user directly supplied the real URL (shubuta.com), not found by MML or either automated pass. Final state: 189/299 (63%) have a City Website value; 110/299 confirmed no official site exists. Population/next-election/officials-roster data collected during research by all agents is not yet merged into this workbook -- future work.</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="8" t="inlineStr">
         <is>
           <t>Municipalities</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="8" t="inlineStr">
         <is>
           <t>Web search (3 parallel research passes); user-supplied correction for Shubuta</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>CivicMirror</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Seeded MS county elected-officeholder backfill (commit a89592ede, issue #36) from the Secretary of State's "County Offices and Directory (2026)" PDF, linked from #36's initial comment. 934 organizations/posts and 1,825 people/memberships across 13 single-county elected office types (Chancery/Circuit Clerk, Tax Assessor, Tax Collector, Coroner, County Court Judge, County Prosecuting Attorney, Sheriff, County Surveyor, Constable, Election Commissioner, Justice Court Judge, County Supervisor) for all 82 counties. Chancery/Circuit Court Judges and District Attorney deliberately held back -- multi-county district offices needing a judicial-district jurisdiction record first (mirrors TX issue #26); appointed offices (per the document's own COUNTY APPOINTED OFFICES section) excluded. Per the workbook's own design, officeholder data lives in the repo data files, not this sheet -- see the Counties sheet Notes column and issue #36/#41 for details. Also substantially answers sub-issue #41 (Judiciary) for the county-court layer.</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Counties, Sources</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Mississippi Secretary of State, County Offices and Directory (2026)</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
         <is>
           <t>CivicMirror</t>
         </is>

</xml_diff>